<commit_message>
feat: agrega funcion para obtener el excel de prestamos
</commit_message>
<xml_diff>
--- a/templates/prestamos_historial.xlsx
+++ b/templates/prestamos_historial.xlsx
@@ -6,7 +6,7 @@
     <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="prestamos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <calcPr/>
   <extLst>
@@ -37,9 +37,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <sz val="11.000000"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12.000000"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
@@ -67,7 +74,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -568,26 +575,26 @@
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="17.28125"/>
-    <col customWidth="1" min="2" max="2" width="15.140625"/>
-    <col customWidth="1" min="3" max="3" width="16.140625"/>
-    <col customWidth="1" min="4" max="4" width="11.57421875"/>
+    <col customWidth="1" min="2" max="2" width="18.28125"/>
+    <col customWidth="1" min="3" max="3" width="20.140625"/>
+    <col customWidth="1" min="4" max="4" width="12.140625"/>
     <col customWidth="1" min="5" max="5" width="11.7109375"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14.25">
-      <c r="A1" t="s">
+    <row r="1" ht="16.5">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
     </row>

</xml_diff>